<commit_message>
Add 거래처코드, 고객코드, 진료과목명 columns to input/output and rebuild exe
</commit_message>
<xml_diff>
--- a/input/A.xlsx
+++ b/input/A.xlsx
@@ -413,102 +413,147 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>거래처코드</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>거래처명</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>시도명</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>시군구명</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>도로명주소</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>전화번호</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>고객코드</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
         <is>
           <t>고객명</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>진료과목명</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>A001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>가톨릭대학교서울성모병원</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>서울특별시</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>서대문구</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>서울특별시 서대문구 연세로 50-1</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>02-1234-5678</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>C001</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
         <is>
           <t>홍길동</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>내과</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>A002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>ABC병원</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>경기도</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>수원시</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>경기도 수원시 영통구</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>031-1899-9542</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>C002</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>김철수</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>정형외과</t>
         </is>
       </c>
     </row>

</xml_diff>